<commit_message>
update docs for sprint 3
</commit_message>
<xml_diff>
--- a/docs/acceptance-tests.xlsx
+++ b/docs/acceptance-tests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ostap\School_Files\Year_3\room-food\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vikto\Documents\HTL\3IHIF\WMC\room-food-docs\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC0B958E-CEE2-464C-87FA-AFAE74E873D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E65FBFC-9B83-4504-9054-7875ABA082B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{8D6859AF-9A25-468C-BEF1-C20AEB03BB66}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{8D6859AF-9A25-468C-BEF1-C20AEB03BB66}"/>
   </bookViews>
   <sheets>
     <sheet name="All Tests" sheetId="1" r:id="rId1"/>
@@ -232,9 +232,6 @@
     <t>Miscellaneous</t>
   </si>
   <si>
-    <t>The user should the means to customize their profile. Including, first name, last name, DOB and profile picture. All the changes should be visible and persistent.</t>
-  </si>
-  <si>
     <t>The users should be able to edits meals they have access to.</t>
   </si>
   <si>
@@ -265,9 +262,6 @@
     <t>If the user requests to delete his account and completely remove it from the database.</t>
   </si>
   <si>
-    <t>logout button which logs a user out of his account .</t>
-  </si>
-  <si>
     <t>When the user signs up the password gets hashed and salted before getting added to the database, password stored in the database should not be readable without the method to decrypt them.</t>
   </si>
   <si>
@@ -287,6 +281,12 @@
   </si>
   <si>
     <t>satisfy criteria of #84 and #85.</t>
+  </si>
+  <si>
+    <t>The user should have the means to customize their profile. Including, first name, last name, DOB and profile picture. All the changes should be visible and persistent.</t>
+  </si>
+  <si>
+    <t>Logout button which logs a user out of their account.</t>
   </si>
 </sst>
 </file>
@@ -342,17 +342,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1011,7 +1010,7 @@
         <v>61</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1022,7 +1021,7 @@
         <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1033,7 +1032,7 @@
         <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1044,7 +1043,7 @@
         <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1055,7 +1054,7 @@
         <v>52</v>
       </c>
       <c r="C6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1066,7 +1065,7 @@
         <v>45</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1077,7 +1076,7 @@
         <v>46</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1088,7 +1087,7 @@
         <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1099,7 +1098,7 @@
         <v>48</v>
       </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1109,8 +1108,8 @@
       <c r="B11" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>65</v>
+      <c r="C11" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1121,7 +1120,7 @@
         <v>49</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1132,7 +1131,7 @@
         <v>50</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>64</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1143,7 +1142,7 @@
         <v>59</v>
       </c>
       <c r="C14" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1154,7 +1153,7 @@
         <v>53</v>
       </c>
       <c r="C15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1165,7 +1164,7 @@
         <v>54</v>
       </c>
       <c r="C16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1176,7 +1175,7 @@
         <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1187,7 +1186,7 @@
         <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1198,7 +1197,7 @@
         <v>57</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1209,7 +1208,7 @@
         <v>60</v>
       </c>
       <c r="C20" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>